<commit_message>
1 commit equivale a cerca de 15 arquivos alterados.´ç
</commit_message>
<xml_diff>
--- a/resources/templates/pauta-geral-template.xlsx
+++ b/resources/templates/pauta-geral-template.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2024-2025\PASTA DAS PAUTAS\PAUTAS ANTIGAS IPIKK\PAUTAS DE INF. 22-23\MINI-PAUTAS DO IIIª-INFORM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell User\Desktop\sistema-escolar2\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="405" yWindow="75" windowWidth="12240" windowHeight="5580"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8205"/>
   </bookViews>
   <sheets>
     <sheet name="INF" sheetId="40" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -255,7 +255,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -4563,8 +4563,8 @@
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>43</xdr:col>
-      <xdr:colOff>157443</xdr:colOff>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>195543</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>133071</xdr:rowOff>
     </xdr:to>
@@ -4615,7 +4615,7 @@
         <xdr:cNvPr id="7" name="Imagem 6" descr="C:\Users\Ahm@d N'landu\Desktop\IMPNV  2037\Logotipo do IMPNV - 2037.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3566D971-9F32-4777-83C0-2EE7CA474EA5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3566D971-9F32-4777-83C0-2EE7CA474EA5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4656,7 +4656,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Escritório">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4694,7 +4694,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Escritório">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4766,7 +4766,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Escritório">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4944,64 +4944,14 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.28515625" style="21" customWidth="1"/>
-    <col min="2" max="2" width="7" style="21" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" style="21" customWidth="1"/>
     <col min="3" max="3" width="37.42578125" style="21" customWidth="1"/>
     <col min="4" max="4" width="3.28515625" style="21" customWidth="1"/>
-    <col min="5" max="5" width="1.5703125" style="21" customWidth="1"/>
-    <col min="6" max="6" width="1.42578125" style="21" customWidth="1"/>
+    <col min="5" max="6" width="2.5703125" style="21" customWidth="1"/>
     <col min="7" max="7" width="0.42578125" style="21" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="2.5703125" style="21" customWidth="1"/>
-    <col min="9" max="10" width="2.7109375" style="21" customWidth="1"/>
-    <col min="11" max="11" width="2.5703125" style="21" customWidth="1"/>
-    <col min="12" max="12" width="2" style="21" customWidth="1"/>
-    <col min="13" max="13" width="1.42578125" style="21" customWidth="1"/>
-    <col min="14" max="14" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="15" max="18" width="2.42578125" style="21" customWidth="1"/>
-    <col min="19" max="20" width="1.7109375" style="21" customWidth="1"/>
-    <col min="21" max="21" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="22" max="23" width="2.7109375" style="21" customWidth="1"/>
-    <col min="24" max="25" width="2.5703125" style="21" customWidth="1"/>
-    <col min="26" max="26" width="1.7109375" style="21" customWidth="1"/>
-    <col min="27" max="27" width="1.42578125" style="21" customWidth="1"/>
-    <col min="28" max="28" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="29" max="31" width="2.7109375" style="21" customWidth="1"/>
-    <col min="32" max="32" width="2.5703125" style="21" customWidth="1"/>
-    <col min="33" max="34" width="1.5703125" style="21" customWidth="1"/>
-    <col min="35" max="35" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="36" max="38" width="2.7109375" style="21" customWidth="1"/>
-    <col min="39" max="39" width="2.42578125" style="21" customWidth="1"/>
-    <col min="40" max="41" width="1.5703125" style="21" customWidth="1"/>
-    <col min="42" max="42" width="2.7109375" style="21" customWidth="1"/>
-    <col min="43" max="44" width="2.7109375" style="9" customWidth="1"/>
-    <col min="45" max="45" width="2.42578125" style="9" customWidth="1"/>
-    <col min="46" max="46" width="2.5703125" style="21" customWidth="1"/>
-    <col min="47" max="47" width="1.5703125" style="21" customWidth="1"/>
-    <col min="48" max="48" width="3.140625" style="21" customWidth="1"/>
-    <col min="49" max="50" width="2.7109375" style="21" customWidth="1"/>
-    <col min="51" max="51" width="2.5703125" style="21" customWidth="1"/>
-    <col min="52" max="52" width="1.7109375" style="21" customWidth="1"/>
-    <col min="53" max="53" width="1.42578125" style="21" customWidth="1"/>
-    <col min="54" max="54" width="2.28515625" style="21" hidden="1" customWidth="1"/>
-    <col min="55" max="57" width="2.7109375" style="21" customWidth="1"/>
-    <col min="58" max="58" width="2.42578125" style="21" customWidth="1"/>
-    <col min="59" max="59" width="1.5703125" style="21" customWidth="1"/>
-    <col min="60" max="60" width="1.42578125" style="21" customWidth="1"/>
-    <col min="61" max="61" width="2.28515625" style="21" hidden="1" customWidth="1"/>
-    <col min="62" max="62" width="2.42578125" style="21" customWidth="1"/>
-    <col min="63" max="65" width="2.7109375" style="21" customWidth="1"/>
-    <col min="66" max="67" width="1.7109375" style="21" customWidth="1"/>
-    <col min="68" max="68" width="2.42578125" style="21" customWidth="1"/>
-    <col min="69" max="71" width="2.5703125" style="21" customWidth="1"/>
-    <col min="72" max="73" width="1.7109375" style="21" customWidth="1"/>
-    <col min="74" max="74" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="75" max="76" width="2.7109375" style="21" customWidth="1"/>
-    <col min="77" max="77" width="3.140625" style="21" customWidth="1"/>
-    <col min="78" max="78" width="2.5703125" style="21" customWidth="1"/>
-    <col min="79" max="80" width="1.7109375" style="21" customWidth="1"/>
-    <col min="81" max="81" width="2.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="82" max="83" width="2.7109375" style="21" customWidth="1"/>
-    <col min="84" max="84" width="3.140625" style="21" customWidth="1"/>
-    <col min="85" max="85" width="2.42578125" style="21" customWidth="1"/>
+    <col min="8" max="42" width="5.7109375" style="21" customWidth="1"/>
+    <col min="43" max="45" width="5.7109375" style="9" customWidth="1"/>
+    <col min="46" max="85" width="5.7109375" style="21" customWidth="1"/>
     <col min="86" max="86" width="7.5703125" style="21" bestFit="1" customWidth="1"/>
     <col min="87" max="87" width="10.85546875" style="21" customWidth="1"/>
     <col min="88" max="88" width="9.140625" style="21" customWidth="1"/>

</xml_diff>